<commit_message>
Correction et amélioration du nouvel export Excel multi-onglet des formations/sessions/séances.
</commit_message>
<xml_diff>
--- a/module/Formation/resources/formation_stats_export_v2.xlsx
+++ b/module/Formation/resources/formation_stats_export_v2.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="DATA_FORM" sheetId="1" state="visible" r:id="rId2"/>
@@ -27,7 +27,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="35">
+  <si>
+    <t xml:space="preserve">module_libelle</t>
+  </si>
   <si>
     <t xml:space="preserve">formation_id</t>
   </si>
@@ -524,7 +527,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" recordCount="1" createdVersion="3">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:T68" sheet="DATA_FORM"/>
+    <worksheetSource ref="B1:U68" sheet="DATA_FORM"/>
   </cacheSource>
   <cacheFields count="20">
     <cacheField name="formation_id" numFmtId="0">
@@ -787,28 +790,29 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T68"/>
-  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:U68"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="121.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="23.54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22.82"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="19.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="20.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="9.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="18.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="0" width="15.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="12.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="18.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="17.67"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="22.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="31.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="30.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="23.54"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="22.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="19.91"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="20.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="9.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="18.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="16" style="0" width="15.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="12.27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="18.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="17.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="22.69"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -872,349 +876,352 @@
       <c r="T1" s="0" t="s">
         <v>19</v>
       </c>
+      <c r="U1" s="0" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="B2" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="G2" s="1"/>
-      <c r="O2" s="2"/>
+      <c r="C2" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="H2" s="1"/>
       <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G3" s="1"/>
-      <c r="O3" s="2"/>
+      <c r="H3" s="1"/>
       <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G4" s="1"/>
-      <c r="O4" s="2"/>
+      <c r="H4" s="1"/>
       <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G5" s="1"/>
-      <c r="O5" s="2"/>
+      <c r="H5" s="1"/>
       <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G6" s="1"/>
-      <c r="O6" s="2"/>
+      <c r="H6" s="1"/>
       <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G7" s="1"/>
-      <c r="O7" s="2"/>
+      <c r="H7" s="1"/>
       <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G8" s="1"/>
-      <c r="O8" s="2"/>
+      <c r="H8" s="1"/>
       <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G9" s="1"/>
-      <c r="O9" s="2"/>
+      <c r="H9" s="1"/>
       <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G10" s="1"/>
-      <c r="O10" s="2"/>
+      <c r="H10" s="1"/>
       <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G11" s="1"/>
-      <c r="O11" s="2"/>
+      <c r="H11" s="1"/>
       <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G12" s="1"/>
-      <c r="O12" s="2"/>
+      <c r="H12" s="1"/>
       <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G13" s="1"/>
-      <c r="O13" s="2"/>
+      <c r="H13" s="1"/>
       <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G14" s="1"/>
-      <c r="O14" s="2"/>
+      <c r="H14" s="1"/>
       <c r="P14" s="2"/>
+      <c r="Q14" s="2"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G15" s="1"/>
-      <c r="O15" s="2"/>
+      <c r="H15" s="1"/>
       <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O16" s="2"/>
       <c r="P16" s="2"/>
+      <c r="Q16" s="2"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O17" s="2"/>
       <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="O18" s="2"/>
+      <c r="E18" s="1"/>
+      <c r="H18" s="1"/>
       <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="O19" s="2"/>
+      <c r="E19" s="1"/>
+      <c r="H19" s="1"/>
       <c r="P19" s="2"/>
+      <c r="Q19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G20" s="1"/>
-      <c r="O20" s="2"/>
+      <c r="H20" s="1"/>
       <c r="P20" s="2"/>
+      <c r="Q20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G21" s="1"/>
-      <c r="O21" s="2"/>
+      <c r="H21" s="1"/>
       <c r="P21" s="2"/>
+      <c r="Q21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="O22" s="2"/>
+      <c r="E22" s="1"/>
+      <c r="H22" s="1"/>
       <c r="P22" s="2"/>
+      <c r="Q22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="O23" s="2"/>
+      <c r="E23" s="1"/>
+      <c r="H23" s="1"/>
       <c r="P23" s="2"/>
+      <c r="Q23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="O24" s="2"/>
+      <c r="E24" s="1"/>
+      <c r="H24" s="1"/>
       <c r="P24" s="2"/>
+      <c r="Q24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="O25" s="2"/>
+      <c r="E25" s="1"/>
+      <c r="H25" s="1"/>
       <c r="P25" s="2"/>
+      <c r="Q25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G26" s="1"/>
-      <c r="O26" s="2"/>
+      <c r="H26" s="1"/>
       <c r="P26" s="2"/>
+      <c r="Q26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G27" s="1"/>
-      <c r="O27" s="2"/>
+      <c r="H27" s="1"/>
       <c r="P27" s="2"/>
+      <c r="Q27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G28" s="1"/>
-      <c r="O28" s="2"/>
+      <c r="H28" s="1"/>
       <c r="P28" s="2"/>
+      <c r="Q28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G29" s="1"/>
-      <c r="O29" s="2"/>
+      <c r="H29" s="1"/>
       <c r="P29" s="2"/>
+      <c r="Q29" s="2"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O30" s="2"/>
       <c r="P30" s="2"/>
+      <c r="Q30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O31" s="2"/>
       <c r="P31" s="2"/>
+      <c r="Q31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O32" s="2"/>
       <c r="P32" s="2"/>
+      <c r="Q32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G33" s="1"/>
-      <c r="O33" s="2"/>
+      <c r="H33" s="1"/>
       <c r="P33" s="2"/>
+      <c r="Q33" s="2"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G34" s="1"/>
-      <c r="O34" s="2"/>
+      <c r="H34" s="1"/>
       <c r="P34" s="2"/>
+      <c r="Q34" s="2"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G35" s="1"/>
-      <c r="O35" s="2"/>
+      <c r="H35" s="1"/>
       <c r="P35" s="2"/>
+      <c r="Q35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O36" s="2"/>
       <c r="P36" s="2"/>
+      <c r="Q36" s="2"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O37" s="2"/>
       <c r="P37" s="2"/>
+      <c r="Q37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O38" s="2"/>
       <c r="P38" s="2"/>
+      <c r="Q38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G39" s="1"/>
-      <c r="O39" s="2"/>
+      <c r="H39" s="1"/>
       <c r="P39" s="2"/>
+      <c r="Q39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O40" s="2"/>
       <c r="P40" s="2"/>
+      <c r="Q40" s="2"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O41" s="2"/>
       <c r="P41" s="2"/>
+      <c r="Q41" s="2"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O42" s="2"/>
       <c r="P42" s="2"/>
+      <c r="Q42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="O43" s="2"/>
       <c r="P43" s="2"/>
+      <c r="Q43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G44" s="1"/>
-      <c r="O44" s="2"/>
+      <c r="H44" s="1"/>
       <c r="P44" s="2"/>
+      <c r="Q44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G45" s="1"/>
-      <c r="O45" s="2"/>
+      <c r="H45" s="1"/>
       <c r="P45" s="2"/>
+      <c r="Q45" s="2"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G46" s="1"/>
-      <c r="O46" s="2"/>
+      <c r="H46" s="1"/>
       <c r="P46" s="2"/>
+      <c r="Q46" s="2"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G47" s="1"/>
-      <c r="O47" s="2"/>
+      <c r="H47" s="1"/>
       <c r="P47" s="2"/>
+      <c r="Q47" s="2"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G48" s="1"/>
-      <c r="O48" s="2"/>
+      <c r="H48" s="1"/>
       <c r="P48" s="2"/>
+      <c r="Q48" s="2"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G49" s="1"/>
-      <c r="O49" s="2"/>
+      <c r="H49" s="1"/>
       <c r="P49" s="2"/>
-      <c r="T49" s="1"/>
+      <c r="Q49" s="2"/>
+      <c r="U49" s="1"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G50" s="1"/>
-      <c r="O50" s="2"/>
+      <c r="H50" s="1"/>
       <c r="P50" s="2"/>
-      <c r="T50" s="1"/>
+      <c r="Q50" s="2"/>
+      <c r="U50" s="1"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G51" s="1"/>
-      <c r="O51" s="2"/>
+      <c r="H51" s="1"/>
       <c r="P51" s="2"/>
-      <c r="T51" s="1"/>
+      <c r="Q51" s="2"/>
+      <c r="U51" s="1"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G52" s="1"/>
-      <c r="O52" s="2"/>
+      <c r="H52" s="1"/>
       <c r="P52" s="2"/>
+      <c r="Q52" s="2"/>
     </row>
     <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G53" s="1"/>
-      <c r="O53" s="2"/>
+      <c r="H53" s="1"/>
       <c r="P53" s="2"/>
+      <c r="Q53" s="2"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G54" s="1"/>
-      <c r="O54" s="2"/>
+      <c r="H54" s="1"/>
       <c r="P54" s="2"/>
+      <c r="Q54" s="2"/>
     </row>
     <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D55" s="1"/>
-      <c r="O55" s="2"/>
+      <c r="E55" s="1"/>
       <c r="P55" s="2"/>
-      <c r="T55" s="1"/>
+      <c r="Q55" s="2"/>
+      <c r="U55" s="1"/>
     </row>
     <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D56" s="1"/>
-      <c r="O56" s="2"/>
+      <c r="E56" s="1"/>
       <c r="P56" s="2"/>
+      <c r="Q56" s="2"/>
     </row>
     <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D57" s="1"/>
-      <c r="O57" s="2"/>
+      <c r="E57" s="1"/>
       <c r="P57" s="2"/>
+      <c r="Q57" s="2"/>
     </row>
     <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D58" s="1"/>
-      <c r="O58" s="2"/>
+      <c r="E58" s="1"/>
       <c r="P58" s="2"/>
+      <c r="Q58" s="2"/>
     </row>
     <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G59" s="1"/>
-      <c r="O59" s="2"/>
+      <c r="H59" s="1"/>
       <c r="P59" s="2"/>
+      <c r="Q59" s="2"/>
     </row>
     <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G60" s="1"/>
-      <c r="O60" s="2"/>
+      <c r="H60" s="1"/>
       <c r="P60" s="2"/>
+      <c r="Q60" s="2"/>
     </row>
     <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G61" s="1"/>
-      <c r="O61" s="2"/>
+      <c r="H61" s="1"/>
       <c r="P61" s="2"/>
+      <c r="Q61" s="2"/>
     </row>
     <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G62" s="1"/>
-      <c r="O62" s="2"/>
+      <c r="H62" s="1"/>
       <c r="P62" s="2"/>
+      <c r="Q62" s="2"/>
     </row>
     <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G63" s="1"/>
-      <c r="O63" s="2"/>
+      <c r="H63" s="1"/>
       <c r="P63" s="2"/>
-      <c r="T63" s="1"/>
+      <c r="Q63" s="2"/>
+      <c r="U63" s="1"/>
     </row>
     <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G64" s="1"/>
-      <c r="O64" s="2"/>
+      <c r="H64" s="1"/>
       <c r="P64" s="2"/>
+      <c r="Q64" s="2"/>
     </row>
     <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G65" s="1"/>
-      <c r="O65" s="2"/>
+      <c r="H65" s="1"/>
       <c r="P65" s="2"/>
+      <c r="Q65" s="2"/>
     </row>
     <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G66" s="1"/>
-      <c r="O66" s="2"/>
+      <c r="H66" s="1"/>
       <c r="P66" s="2"/>
-      <c r="T66" s="1"/>
+      <c r="Q66" s="2"/>
+      <c r="U66" s="1"/>
     </row>
     <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G67" s="1"/>
-      <c r="O67" s="2"/>
+      <c r="H67" s="1"/>
       <c r="P67" s="2"/>
-      <c r="T67" s="1"/>
+      <c r="Q67" s="2"/>
+      <c r="U67" s="1"/>
     </row>
     <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="G68" s="1"/>
-      <c r="O68" s="2"/>
+      <c r="H68" s="1"/>
       <c r="P68" s="2"/>
-      <c r="T68" s="1"/>
+      <c r="Q68" s="2"/>
+      <c r="U68" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1233,7 +1240,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:T5"/>
-  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3"/>
@@ -1253,7 +1260,7 @@
       <c r="O1" s="4"/>
       <c r="P1" s="5"/>
       <c r="Q1" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="R1" s="7"/>
       <c r="S1" s="7"/>
@@ -1261,114 +1268,114 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="I2" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="I2" s="10" t="s">
-        <v>6</v>
-      </c>
       <c r="J2" s="10" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L2" s="10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="M2" s="10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="O2" s="10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="P2" s="10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q2" s="11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="R2" s="12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="S2" s="12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="T2" s="13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C3" s="15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E3" s="16" t="n">
         <v>1</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H3" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I3" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J3" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K3" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L3" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N3" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O3" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P3" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q3" s="17"/>
       <c r="R3" s="18"/>
@@ -1381,40 +1388,40 @@
       <c r="C4" s="21"/>
       <c r="D4" s="21"/>
       <c r="E4" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I4" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J4" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K4" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="L4" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M4" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N4" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="O4" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="P4" s="16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q4" s="17"/>
       <c r="R4" s="18"/>
@@ -1423,7 +1430,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="22" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="23"/>
       <c r="C5" s="23"/>
@@ -1462,7 +1469,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H1002"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.43"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="53.38"/>
@@ -1476,28 +1483,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B1" s="0" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C1" s="0" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D1" s="0" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E1" s="0" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F1" s="0" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G1" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H1" s="0" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1505,7 +1512,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H2" s="2"/>
     </row>
@@ -4528,7 +4535,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -4546,7 +4553,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>